<commit_message>
docs(validation): record 2026-07-13 live market observations and execution decision review
docs(validation): record 2026-07-13 live market observations and execution decision review

- Added live market validation observations
- Recorded multi-timeframe KRONOS behaviour across equities and commodities
- Documented repeated BUY READY execution-chart observations
- Updated validation evidence for post-market engineering review
- No trading logic or Pine implementation changes
</commit_message>
<xml_diff>
--- a/data/trades/KRONOS_TRADE_LEDGER.xlsx
+++ b/data/trades/KRONOS_TRADE_LEDGER.xlsx
@@ -129,7 +129,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>8</t>
         </is>
       </c>
     </row>
@@ -141,7 +141,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>8</t>
         </is>
       </c>
     </row>
@@ -1087,8 +1087,944 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>KR-OBS-20260713-001</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Gold Futures</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>MCX</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Multi-Timeframe</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Daily Screenshot Review</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>ChatGPT Screenshot Review</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>KR-SCR-20260713-001</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>assets/validation/observations/KR-SCR-20260713-001-gold-futures.png</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Higher timeframe bearish. Execution timeframe weak. Observation only.</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Observation only</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>KR-OBS-20260713-002</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Silver Futures</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>MCX</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Multi-Timeframe</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Daily Screenshot Review</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>ChatGPT Screenshot Review</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>KR-SCR-20260713-002</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>assets/validation/observations/KR-SCR-20260713-002-silver-futures.png</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Bearish structure. Momentum fading. Observation only.</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Observation only</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>KR-OBS-20260713-003</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Copper Futures</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>MCX</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Multi-Timeframe</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Daily Screenshot Review</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>ChatGPT Screenshot Review</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>KR-SCR-20260713-003</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>assets/validation/observations/KR-SCR-20260713-003-copper-futures.png</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Healthy higher-timeframe structure. Execution momentum exhausted. Watch Long. No trade.</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Watch Long; no trade</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>KR-OBS-20260713-004</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Natural Gas Futures</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>MCX</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Multi-Timeframe</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Daily Screenshot Review</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>ChatGPT Screenshot Review</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>KR-SCR-20260713-004</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>assets/validation/observations/KR-SCR-20260713-004-natural-gas-futures.png</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>Higher-timeframe bearish structure remains intact. Execution timeframe is already extended. No entry because the move is considered late. Await pullback before considering any short setup.</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Watch Short</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>KR-OBS-20260713-005</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>MARUTI</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>1H execution chart reviewed with Weekly/Daily/4H context</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Conflicting Evidence; Decision; UI / Presentation; Research Hypothesis</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>ChatGPT Screenshot Review</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>KR-SCR-20260713-005</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>assets/validation/observations/KR-SCR-20260713-005-maruti-1h.png</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Weekly Neutral / awaiting trend confirmation; Daily Neutral / awaiting trend confirmation; 4H Bullish but weak; 1H Bearish local state</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>4H weak context noted; 1H local evidence supported short setup</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>4H testing acceptance</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>4H exhausted momentum; 1H high-confidence local bearish state</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Local 1H state supported short setup</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>SELL READY displayed on 1H execution chart</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>KRONOS displayed SELL READY on the 1H execution chart. Higher-timeframe context was mixed: Weekly Neutral / awaiting confirmation, Daily Neutral / awaiting confirmation, 4H Bullish but weak with testing acceptance and exhausted momentum, while 1H showed bearish local state with high confidence. Partial Agreement: local 1H state supported a short setup, but complete multi-timeframe structure did not support an unambiguous consolidated SELL READY instruction. Key finding: execution chart appears to expose a local execution-timeframe decision rather than the final consolidated multi-timeframe KRONOS decision. Hypothesis: KR-705 may be displaying a local KR-370/KR-380 output computed in the chart timeframe without a separate final multi-timeframe decision contract. Affected engines: KR-300, KR-340, KR-350, KR-360, KR-370, KR-380, KR-705. Priority: High. Status: Confirmed for architectural review.</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>Audit current source and implement a consolidated execution-chart decision contract. No Pine change during market hours.</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>KR-OBS-20260713-006</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Bajaj Auto Limited</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>1W / 1D / 4H / 1H</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Execution Chart Decision Principle; Conflicting Evidence; UI / Presentation</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>ChatGPT Screenshot Review</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>KR-SCR-20260713-006</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>assets/validation/observations/KR-SCR-20260713-001.png</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Weekly Bullish; Daily Neutral; 4H Neutral; 1H Bullish</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Weekly WATCH LONG; Daily AVOID / WAITING; 4H AVOID / WAITING; 1H BUY READY with Entry: NO TRIGGER</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>The execution chart displayed BUY READY while higher confirmation timeframes had not yet reached a consolidated bullish decision. Weekly: Trend Bullish, Decision WATCH LONG. Daily: Trend Neutral, Decision AVOID, Status WAITING. 4H: Trend Neutral, Decision AVOID, Status WAITING. 1H: Trend Bullish, Decision BUY READY, Entry NO TRIGGER. Validation note: the execution chart appears to present local execution-timeframe readiness rather than the final consolidated KRONOS decision. Impact: potential trader confusion regarding whether BUY READY represents local readiness or consolidated multi-timeframe readiness.</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>Record for architectural review after market hours. No Pine changes. No implementation changes. No trading decision based solely on this observation.</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>KR-OBS-20260713-007</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>One 97 Communications Ltd. (Paytm)</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>1W / 1D / 4H / 1H</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Execution Chart Decision Principle; Conflicting Evidence; UI / Presentation</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>ChatGPT Screenshot Review</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>KR-SCR-20260713-007</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>assets/validation/observations/KR-SCR-20260713-002.png</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Weekly Neutral; Daily Bullish; 4H Bullish; 1H Bullish</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>Weekly AVOID; Daily WATCH LONG with Entry NO TRIGGER; 4H WATCH LONG with Confidence 42 (Developing); 1H BUY READY with Confidence 86 (Exceptional) and Entry NO TRIGGER</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>The execution chart displayed BUY READY while higher confirmation timeframes remained in WATCH LONG rather than BUY READY. Weekly: Trend Neutral, Decision AVOID. Daily: Trend Bullish, Decision WATCH LONG, Entry NO TRIGGER. 4H: Trend Bullish, Decision WATCH LONG, Confidence 42 (Developing). 1H: Trend Bullish, Decision BUY READY, Confidence 86 (Exceptional), Entry NO TRIGGER. Validation note: this matches an earlier observation where the execution chart appears to present local execution readiness before higher-timeframe decision panels have reached an equivalent readiness state. Impact: additional evidence for reviewing whether BUY READY should represent a fully consolidated KRONOS decision across all required timeframes.</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>Record for post-market architectural review only. No implementation changes during market hours.</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>KR-OBS-20260713-008</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>HCL Technologies Ltd.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>1W / 1D / 4H / 1H</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Execution Chart Decision Principle; Conflicting Evidence; UI / Presentation</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>ChatGPT Screenshot Review</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>KR-SCR-20260713-008</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>assets/validation/observations/KR-SCR-20260713-003.png</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Weekly Bearish; Daily Bearish; 4H Bearish; 1H Bullish</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Weekly/Daily/4H Acceptance Pending</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Weekly WATCH SHORT; Daily WATCH SHORT; 4H WATCH SHORT; 1H BUY READY with Confidence 90 (Exceptional) and Entry NO TRIGGER</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>The execution chart displayed BUY READY while Weekly, Daily, and 4H remained in WATCH SHORT with Acceptance Pending. Weekly: Trend Bearish, Decision WATCH SHORT. Daily: Trend Bearish, Decision WATCH SHORT. 4H: Trend Bearish, Decision WATCH SHORT. 1H: Trend Bullish, Decision BUY READY, Confidence 90 (Exceptional), Entry NO TRIGGER. Validation note: this is another example where the execution timeframe reports local bullish readiness before higher-timeframe panels transition to a consolidated bullish decision. Impact: additional evidence for reviewing whether BUY READY on the execution chart should represent local execution readiness or the final consolidated KRONOS decision.</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>Record for post-market architectural review. No implementation changes during market hours.</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:W1"/>
+  <autoFilter ref="A1:W9"/>
 </worksheet>
 </file>
 
@@ -1171,8 +2107,504 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>KR-SCR-20260713-001</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Gold Futures</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>MCX</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Multi-Timeframe</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>assets/validation/observations/KR-SCR-20260713-001-gold-futures.png</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>KR-OBS-20260713-001</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>TradingView Screenshot Review</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Higher timeframe bearish; execution timeframe weak.</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>KR-SCR-20260713-002</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Silver Futures</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>MCX</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Multi-Timeframe</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>assets/validation/observations/KR-SCR-20260713-002-silver-futures.png</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>KR-OBS-20260713-002</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>TradingView Screenshot Review</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Bearish structure; momentum fading.</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>KR-SCR-20260713-003</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Copper Futures</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>MCX</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Multi-Timeframe</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>assets/validation/observations/KR-SCR-20260713-003-copper-futures.png</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>KR-OBS-20260713-003</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>TradingView Screenshot Review</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Healthy higher-timeframe structure; execution momentum exhausted; Watch Long; no trade.</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>KR-SCR-20260713-004</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Natural Gas Futures</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>MCX</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Multi-Timeframe</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>assets/validation/observations/KR-SCR-20260713-004-natural-gas-futures.png</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>KR-OBS-20260713-004</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>TradingView Screenshot Review</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Higher-timeframe bearish structure intact; execution extended; late move; await pullback before short setup.</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>KR-SCR-20260713-005</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>MARUTI</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>1H execution chart reviewed with Weekly/Daily/4H context</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>assets/validation/observations/KR-SCR-20260713-005-maruti-1h.png</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>KR-OBS-20260713-005</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>TradingView Screenshot Review</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>MARUTI SELL READY display reviewed as conflicting evidence / UI presentation / research hypothesis. Partial Agreement. Priority High. Confirmed for architectural review.</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>KR-SCR-20260713-006</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Bajaj Auto Limited</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>1W / 1D / 4H / 1H</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>assets/validation/observations/KR-SCR-20260713-001.png</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>KR-OBS-20260713-006</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>TradingView Screenshot Review</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Execution chart displayed BUY READY while higher confirmation timeframes were not consolidated bullish. Architectural review record; no trade decision.</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>KR-SCR-20260713-007</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>One 97 Communications Ltd. (Paytm)</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>1W / 1D / 4H / 1H</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>assets/validation/observations/KR-SCR-20260713-002.png</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>KR-OBS-20260713-007</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>TradingView Screenshot Review</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Execution chart displayed BUY READY while higher confirmation timeframes remained WATCH LONG / AVOID. Architectural review record; no implementation changes during market hours.</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>KR-SCR-20260713-008</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>HCL Technologies Ltd.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>1W / 1D / 4H / 1H</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>assets/validation/observations/KR-SCR-20260713-003.png</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>KR-OBS-20260713-008</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>TradingView Screenshot Review</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Execution chart displayed BUY READY while Weekly/Daily/4H remained WATCH SHORT with Acceptance Pending. Architectural review record; no implementation changes during market hours.</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L1"/>
+  <autoFilter ref="A1:L9"/>
 </worksheet>
 </file>
 

</xml_diff>